<commit_message>
Moved data, made new analysis ipynb
</commit_message>
<xml_diff>
--- a/contact_correlations/heating_metadata.xlsx
+++ b/contact_correlations/heating_metadata.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74813801-ECC3-4E0F-A756-FD5C06FDEB6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11835"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
   <si>
     <t>filename</t>
   </si>
@@ -104,12 +103,21 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>2024-04-05_C_UHfit</t>
+  </si>
+  <si>
+    <t>2024-03-26_B_UHfit</t>
+  </si>
+  <si>
+    <t>reanalyzed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -142,10 +150,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,8 +434,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H13"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
@@ -434,7 +443,7 @@
     <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -459,8 +468,11 @@
       <c r="H1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -485,8 +497,11 @@
       <c r="H2">
         <v>441</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -511,8 +526,11 @@
       <c r="H3">
         <v>441</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -537,16 +555,19 @@
       <c r="H4">
         <v>441</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="1">
         <v>45377</v>
@@ -563,42 +584,48 @@
       <c r="H5">
         <v>441</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>45377</v>
+      </c>
+      <c r="E6">
+        <v>202.14</v>
+      </c>
+      <c r="F6">
+        <v>169.1</v>
+      </c>
+      <c r="G6">
+        <v>453</v>
+      </c>
+      <c r="H6">
+        <v>441</v>
+      </c>
+      <c r="I6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1">
-        <v>45385</v>
-      </c>
-      <c r="E6">
-        <v>202.14</v>
-      </c>
-      <c r="F6" s="2">
-        <v>151.24763799808576</v>
-      </c>
-      <c r="G6" s="2">
-        <v>405.17551752296185</v>
-      </c>
-      <c r="H6" s="2">
-        <v>394.44239123096287</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="1">
         <v>45385</v>
@@ -615,19 +642,22 @@
       <c r="H7" s="2">
         <v>394.44239123096287</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>45386</v>
+        <v>45385</v>
       </c>
       <c r="E8">
         <v>202.14</v>
@@ -641,10 +671,13 @@
       <c r="H8" s="2">
         <v>394.44239123096287</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
@@ -653,85 +686,94 @@
         <v>0</v>
       </c>
       <c r="D9" s="1">
+        <v>45386</v>
+      </c>
+      <c r="E9">
+        <v>202.14</v>
+      </c>
+      <c r="F9" s="2">
+        <v>151.24763799808576</v>
+      </c>
+      <c r="G9" s="2">
+        <v>405.17551752296185</v>
+      </c>
+      <c r="H9" s="2">
+        <v>394.44239123096287</v>
+      </c>
+      <c r="I9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>45387</v>
+      </c>
+      <c r="E10">
+        <v>202.14</v>
+      </c>
+      <c r="F10" s="2">
+        <v>151.24763799808576</v>
+      </c>
+      <c r="G10" s="2">
+        <v>405.17551752296185</v>
+      </c>
+      <c r="H10" s="2">
+        <v>394.44239123096287</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11" s="1">
         <v>45392</v>
       </c>
-      <c r="E9">
-        <v>202.14</v>
-      </c>
-      <c r="F9">
+      <c r="E11">
+        <v>202.14</v>
+      </c>
+      <c r="F11">
         <v>169.1</v>
       </c>
-      <c r="G9">
+      <c r="G11">
         <v>453</v>
       </c>
-      <c r="H9">
+      <c r="H11">
         <v>441</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="I11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>21</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12" s="1">
         <v>45392</v>
-      </c>
-      <c r="E10">
-        <v>202.14</v>
-      </c>
-      <c r="F10">
-        <v>169.1</v>
-      </c>
-      <c r="G10">
-        <v>453</v>
-      </c>
-      <c r="H10">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" s="1">
-        <v>45421</v>
-      </c>
-      <c r="E11">
-        <v>202.14</v>
-      </c>
-      <c r="F11" s="2">
-        <v>151.24763799808576</v>
-      </c>
-      <c r="G11" s="2">
-        <v>405.17551752296185</v>
-      </c>
-      <c r="H11" s="2">
-        <v>394.44239123096287</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1">
-        <v>45422</v>
       </c>
       <c r="E12">
         <v>202.14</v>
@@ -745,31 +787,95 @@
       <c r="H12">
         <v>441</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" s="1">
+        <v>45421</v>
+      </c>
+      <c r="E13">
+        <v>202.14</v>
+      </c>
+      <c r="F13" s="2">
+        <v>151.24763799808576</v>
+      </c>
+      <c r="G13" s="2">
+        <v>405.17551752296185</v>
+      </c>
+      <c r="H13" s="2">
+        <v>394.44239123096287</v>
+      </c>
+      <c r="I13" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>45422</v>
+      </c>
+      <c r="E14">
+        <v>202.14</v>
+      </c>
+      <c r="F14">
+        <v>169.1</v>
+      </c>
+      <c r="G14">
+        <v>453</v>
+      </c>
+      <c r="H14">
+        <v>441</v>
+      </c>
+      <c r="I14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B15" t="s">
         <v>27</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13" s="1">
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
         <v>45422</v>
       </c>
-      <c r="E13">
-        <v>202.14</v>
-      </c>
-      <c r="F13">
+      <c r="E15">
+        <v>202.14</v>
+      </c>
+      <c r="F15">
         <v>169.1</v>
       </c>
-      <c r="G13">
+      <c r="G15">
         <v>453</v>
       </c>
-      <c r="H13">
+      <c r="H15">
         <v>441</v>
+      </c>
+      <c r="I15" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added B and barnu from metadata
</commit_message>
<xml_diff>
--- a/contact_correlations/heating_metadata.xlsx
+++ b/contact_correlations/heating_metadata.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>filename</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>reanalyzed</t>
+  </si>
+  <si>
+    <t>barnu</t>
   </si>
 </sst>
 </file>
@@ -435,15 +438,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -469,10 +473,13 @@
         <v>8</v>
       </c>
       <c r="I1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -497,11 +504,15 @@
       <c r="H2">
         <v>441</v>
       </c>
-      <c r="I2" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2">
+        <f>(F2*G2*H2)^(1/3)</f>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -526,11 +537,15 @@
       <c r="H3">
         <v>441</v>
       </c>
-      <c r="I3" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <f t="shared" ref="I3:I15" si="0">(F3*G3*H3)^(1/3)</f>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -555,11 +570,15 @@
       <c r="H4">
         <v>441</v>
       </c>
-      <c r="I4" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I4">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J4" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -584,11 +603,15 @@
       <c r="H5">
         <v>441</v>
       </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J5" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -613,11 +636,15 @@
       <c r="H6">
         <v>441</v>
       </c>
-      <c r="I6" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -642,11 +669,15 @@
       <c r="H7" s="2">
         <v>394.44239123096287</v>
       </c>
-      <c r="I7" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>289.13796930194775</v>
+      </c>
+      <c r="J7" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -671,11 +702,15 @@
       <c r="H8" s="2">
         <v>394.44239123096287</v>
       </c>
-      <c r="I8" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>289.13796930194775</v>
+      </c>
+      <c r="J8" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -700,11 +735,15 @@
       <c r="H9" s="2">
         <v>394.44239123096287</v>
       </c>
-      <c r="I9" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>289.13796930194775</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -729,11 +768,15 @@
       <c r="H10" s="2">
         <v>394.44239123096287</v>
       </c>
-      <c r="I10" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10">
+        <f t="shared" si="0"/>
+        <v>289.13796930194775</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -758,11 +801,15 @@
       <c r="H11">
         <v>441</v>
       </c>
-      <c r="I11" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I11">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -787,11 +834,15 @@
       <c r="H12">
         <v>441</v>
       </c>
-      <c r="I12" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I12">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -816,11 +867,15 @@
       <c r="H13" s="2">
         <v>394.44239123096287</v>
       </c>
-      <c r="I13" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I13">
+        <f t="shared" si="0"/>
+        <v>289.13796930194775</v>
+      </c>
+      <c r="J13" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -845,11 +900,15 @@
       <c r="H14">
         <v>441</v>
       </c>
-      <c r="I14" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I14">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J14" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -874,7 +933,11 @@
       <c r="H15">
         <v>441</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15">
+        <f t="shared" si="0"/>
+        <v>323.26607711770117</v>
+      </c>
+      <c r="J15" s="3">
         <v>1</v>
       </c>
     </row>

</xml_diff>